<commit_message>
Excel: Kopfzeile mit Bilanz wiederhergestellt, Backup-Muster in .gitignore erweitert
Alle übrigen Korrekturen wurden gemeinsam geprüft und bestätigt;
Original-Excel und data/werderspiele.xlsx sind jetzt inhaltlich identisch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/werderspiele.xlsx
+++ b/data/werderspiele.xlsx
@@ -750,7 +750,11 @@
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
-      <c r="H1" s="12" t="n"/>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>S: 158, U: 103, N: 127</t>
+        </is>
+      </c>
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
@@ -25304,7 +25308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:S184"/>
+  <dimension ref="A1:S184"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.75"/>
   <cols>
     <col width="11.453125" customWidth="1" style="13" min="1" max="1"/>
@@ -25443,6 +25447,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="14" t="inlineStr">
         <is>

</xml_diff>